<commit_message>
diagnostic of fragility metric
</commit_message>
<xml_diff>
--- a/outputs/tables/ame_bootstrap_results.xlsx
+++ b/outputs/tables/ame_bootstrap_results.xlsx
@@ -47,7 +47,7 @@
     <t xml:space="preserve">n_boot_fail</t>
   </si>
   <si>
-    <t xml:space="preserve">Redundant → Fragile</t>
+    <t xml:space="preserve">Redundant -&gt; Fragile</t>
   </si>
   <si>
     <t xml:space="preserve">z_log_median_income</t>
@@ -68,22 +68,22 @@
     <t xml:space="preserve">z_renter_share</t>
   </si>
   <si>
-    <t xml:space="preserve">Redundant → Isolated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redundant → Inundated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redundant → Worse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fragile → Isolated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fragile → Inundated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fragile → Worse</t>
+    <t xml:space="preserve">Redundant -&gt; Isolated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redundant -&gt; Inundated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redundant -&gt; Worse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fragile -&gt; Isolated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fragile -&gt; Inundated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fragile -&gt; Worse</t>
   </si>
 </sst>
 </file>
@@ -878,19 +878,19 @@
         <v>-0.000914768571830827</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0032911574109166</v>
+        <v>0.0034621303118806</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.277947377660086</v>
+        <v>-0.26422130001627</v>
       </c>
       <c r="F14" t="n">
-        <v>0.781052754103902</v>
+        <v>0.791609399065543</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.00680738401130868</v>
+        <v>-0.00842986375950556</v>
       </c>
       <c r="H14" t="n">
-        <v>0.00590037244516919</v>
+        <v>0.00554166729602935</v>
       </c>
       <c r="I14" t="n">
         <v>0.95</v>
@@ -913,19 +913,19 @@
         <v>0.000525490880226845</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00220886028032719</v>
+        <v>0.00257566151339105</v>
       </c>
       <c r="E15" t="n">
-        <v>0.23790136701132</v>
+        <v>0.204021715390311</v>
       </c>
       <c r="F15" t="n">
-        <v>0.811957595228925</v>
+        <v>0.838336529375296</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.0038246774542196</v>
+        <v>-0.00439182485067174</v>
       </c>
       <c r="H15" t="n">
-        <v>0.00453754966483861</v>
+        <v>0.00521172845466085</v>
       </c>
       <c r="I15" t="n">
         <v>0.95</v>
@@ -948,19 +948,19 @@
         <v>0.00771029099369581</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00382902670077424</v>
+        <v>0.00360155460989792</v>
       </c>
       <c r="E16" t="n">
-        <v>2.01364252491025</v>
+        <v>2.14082301362476</v>
       </c>
       <c r="F16" t="n">
-        <v>0.044047078343018</v>
+        <v>0.0322883133546609</v>
       </c>
       <c r="G16" t="n">
-        <v>0.000779496276238455</v>
+        <v>0.00101677815697012</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0147325315072233</v>
+        <v>0.0145715140807224</v>
       </c>
       <c r="I16" t="n">
         <v>0.95</v>
@@ -983,19 +983,19 @@
         <v>-0.0282337318573982</v>
       </c>
       <c r="D17" t="n">
-        <v>0.00354324154724335</v>
+        <v>0.00342666807584707</v>
       </c>
       <c r="E17" t="n">
-        <v>-7.96833393403961</v>
+        <v>-8.23941252332088</v>
       </c>
       <c r="F17" t="n">
-        <v>0.00000000000000160827797131878</v>
+        <v>0.000000000000000173058284517338</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.0349211278030549</v>
+        <v>-0.0340857149667673</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.0218463772573484</v>
+        <v>-0.0213500961320285</v>
       </c>
       <c r="I17" t="n">
         <v>0.95</v>
@@ -1018,19 +1018,19 @@
         <v>-0.0336653447595364</v>
       </c>
       <c r="D18" t="n">
-        <v>0.00437394653064631</v>
+        <v>0.00408001797133297</v>
       </c>
       <c r="E18" t="n">
-        <v>-7.69678927798001</v>
+        <v>-8.25127364537997</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0000000000000139527708984243</v>
+        <v>0.000000000000000156715240209812</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.0425463997968203</v>
+        <v>-0.0409368003634984</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.0254593589103788</v>
+        <v>-0.0258053686962622</v>
       </c>
       <c r="I18" t="n">
         <v>0.95</v>
@@ -1053,19 +1053,19 @@
         <v>0.02313451838478</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0029632617471325</v>
+        <v>0.00312079922456524</v>
       </c>
       <c r="E19" t="n">
-        <v>7.80711268829591</v>
+        <v>7.41301080911508</v>
       </c>
       <c r="F19" t="n">
-        <v>0.00000000000000585129500483862</v>
+        <v>0.000000000000123463818915723</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0179724123112614</v>
+        <v>0.0172110958192586</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0287697167488173</v>
+        <v>0.0295630607241939</v>
       </c>
       <c r="I19" t="n">
         <v>0.95</v>
@@ -1088,19 +1088,19 @@
         <v>0.00380932620214313</v>
       </c>
       <c r="D20" t="n">
-        <v>0.00567602513396819</v>
+        <v>0.00549536079406588</v>
       </c>
       <c r="E20" t="n">
-        <v>0.671125675491852</v>
+        <v>0.693189463784908</v>
       </c>
       <c r="F20" t="n">
-        <v>0.502140471707618</v>
+        <v>0.488190659402193</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.00715882504863775</v>
+        <v>-0.00603569373590915</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0154421517228712</v>
+        <v>0.0154922341432606</v>
       </c>
       <c r="I20" t="n">
         <v>0.95</v>
@@ -1123,19 +1123,19 @@
         <v>-0.00213669230055808</v>
       </c>
       <c r="D21" t="n">
-        <v>0.00394606983295204</v>
+        <v>0.00340947494460633</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.541473514410574</v>
+        <v>-0.626692477660896</v>
       </c>
       <c r="F21" t="n">
-        <v>0.58818124839291</v>
+        <v>0.530860835710009</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.0094836189986915</v>
+        <v>-0.00925908651647135</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0050773660434693</v>
+        <v>0.00405253596790495</v>
       </c>
       <c r="I21" t="n">
         <v>0.95</v>
@@ -1158,19 +1158,19 @@
         <v>0.0172548546495021</v>
       </c>
       <c r="D22" t="n">
-        <v>0.00544485858148129</v>
+        <v>0.00574541342293645</v>
       </c>
       <c r="E22" t="n">
-        <v>3.16901796277835</v>
+        <v>3.00323986792985</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0015295494176796</v>
+        <v>0.00267121801493338</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0083989100320284</v>
+        <v>0.00631413604452782</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0279386007238878</v>
+        <v>0.0289863324688782</v>
       </c>
       <c r="I22" t="n">
         <v>0.95</v>
@@ -1193,19 +1193,19 @@
         <v>-0.0462694160681533</v>
       </c>
       <c r="D23" t="n">
-        <v>0.00481175992131982</v>
+        <v>0.00476629895001862</v>
       </c>
       <c r="E23" t="n">
-        <v>-9.61590287643902</v>
+        <v>-9.7076193821146</v>
       </c>
       <c r="F23" t="n">
-        <v>0.000000000000000000000685056696468512</v>
+        <v>0.0000000000000000000002797955367902</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.0537780734304305</v>
+        <v>-0.0546539841202694</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0357819278977259</v>
+        <v>-0.0376170677587492</v>
       </c>
       <c r="I23" t="n">
         <v>0.95</v>
@@ -1228,19 +1228,19 @@
         <v>-0.0580867431464548</v>
       </c>
       <c r="D24" t="n">
-        <v>0.00567540542788191</v>
+        <v>0.00627246576608368</v>
       </c>
       <c r="E24" t="n">
-        <v>-10.2348182670948</v>
+        <v>-9.26059149824937</v>
       </c>
       <c r="F24" t="n">
-        <v>0.00000000000000000000000138454880326198</v>
+        <v>0.0000000000000000000203302806370077</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.0685374723525503</v>
+        <v>-0.0701203243136977</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.0466776694339676</v>
+        <v>-0.0456221350583177</v>
       </c>
       <c r="I24" t="n">
         <v>0.95</v>
@@ -1263,19 +1263,19 @@
         <v>0.0397623654528539</v>
       </c>
       <c r="D25" t="n">
-        <v>0.00477531873662931</v>
+        <v>0.00465692261742525</v>
       </c>
       <c r="E25" t="n">
-        <v>8.32664114080067</v>
+        <v>8.53833501636281</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0000000000000000831683705367693</v>
+        <v>0.000000000000000013616964045152</v>
       </c>
       <c r="G25" t="n">
-        <v>0.0306676531047223</v>
+        <v>0.0314491421800249</v>
       </c>
       <c r="H25" t="n">
-        <v>0.049250901313192</v>
+        <v>0.0485637013387214</v>
       </c>
       <c r="I25" t="n">
         <v>0.95</v>

</xml_diff>